<commit_message>
Add invoice and packing list number columns to HAWB 5948470682 summary
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E5tGdT1wYCN5r8Rnct91dS
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Quanta_5948470682.xlsx
+++ b/output/HS_Code_Summary_Quanta_5948470682.xlsx
@@ -456,19 +456,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,35 +498,45 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Invoice No.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Packing List No.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>COO</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Quantity (SET)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Net weight (kg)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Unit price (USD)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Customs value (USD)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -548,27 +560,37 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>2215689265</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2026195908</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="G4" s="3" t="n">
         <v>960</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>10.944</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="I4" s="3" t="n">
         <v>20.1</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>7.89</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="K4" s="3" t="n">
         <v>7574.4</v>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Invoice 2215689265 / PL 2026195908 / P/O 4119001585-387 / 1 PLT = 3 CTNS</t>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>P/O 4119001585-387 / 1 PLT = 3 CTNS (PLT.1GE5908)</t>
         </is>
       </c>
     </row>
@@ -590,27 +612,37 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>2215689266</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>2026195909</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="G5" s="3" t="n">
         <v>1600</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="H5" s="3" t="n">
         <v>18.24</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="I5" s="3" t="n">
         <v>42.3</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>7.89</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>12624</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Invoice 2215689266 / PL 2026195909 / P/O 4119001585-426 / 1 PLT = 5 CTNS</t>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>P/O 4119001585-426 / 1 PLT = 5 CTNS (PLT.1GE5909)</t>
         </is>
       </c>
     </row>
@@ -627,20 +659,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="n">
         <v>2560</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>29.184</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>62.4</v>
       </c>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="n">
         <v>20198.4</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>2 PLTS = 8 CTNS</t>
         </is>
@@ -707,15 +741,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A10:L10"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A12:L12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>